<commit_message>
refactor: update fee table schema to support partner management, replace supplier references with partner terminology, and enhance validation logic for fee table imports and price tables
</commit_message>
<xml_diff>
--- a/docs/templates/fee-table-import-template.xlsx
+++ b/docs/templates/fee-table-import-template.xlsx
@@ -671,7 +671,7 @@
         <v>target</v>
       </c>
       <c r="B38" t="str">
-        <v>CUSTOMER | SUPPLIER</v>
+        <v>CUSTOMER | PARTNER</v>
       </c>
     </row>
     <row r="39">
@@ -679,7 +679,7 @@
         <v>scope.objectType</v>
       </c>
       <c r="B39" t="str">
-        <v>SUPPLIER_INTERNAL | SUPPLIER_EXTERNAL | CUSTOMER_INDIVIDUAL | CUSTOMER_BUSINESS</v>
+        <v>PARTNER_INTERNAL | PARTNER_EXTERNAL | CUSTOMER_INDIVIDUAL | CUSTOMER_BUSINESS</v>
       </c>
     </row>
     <row r="40">
@@ -708,26 +708,26 @@
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>enterpriseCode</v>
+        <v>corporateCustomerId</v>
       </c>
       <c r="B43" t="str">
-        <v>Mã DN — bắt buộc khi kind=CUSTOMER_BUSINESS</v>
+        <v>Mã KH DN — bắt buộc khi object_type=CUSTOMER_BUSINESS</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>supplierId</v>
+        <v>partnerId</v>
       </c>
       <c r="B44" t="str">
-        <v>Mã NCC — bắt buộc khi kind=SUPPLIER_EXTERNAL</v>
+        <v>Mã Partner/NCC — bắt buộc khi object_type=PARTNER_EXTERNAL (không fallback)</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>supplierName</v>
+        <v>partnerName</v>
       </c>
       <c r="B45" t="str">
-        <v>Tên NCC (tùy chọn)</v>
+        <v>Tên Partner/NCC (tùy chọn)</v>
       </c>
     </row>
     <row r="46">
@@ -735,7 +735,7 @@
         <v>retailMarkupFactor</v>
       </c>
       <c r="B46" t="str">
-        <v>Hệ số giá khách lẻ (0 = không dùng; &gt;0 chỉ với CUSTOMER_RETAIL markup-only)</v>
+        <v>Hệ số giá khách lẻ (0 = không dùng; &gt;0 chỉ với CUSTOMER_INDIVIDUAL markup-only)</v>
       </c>
     </row>
     <row r="47">
@@ -802,7 +802,7 @@
         <v>target</v>
       </c>
       <c r="B4" t="str">
-        <v>SUPPLIER</v>
+        <v>PARTNER</v>
       </c>
     </row>
     <row r="5">
@@ -810,7 +810,7 @@
         <v>scope.objectType</v>
       </c>
       <c r="B5" t="str">
-        <v>SUPPLIER_EXTERNAL</v>
+        <v>PARTNER_EXTERNAL</v>
       </c>
     </row>
     <row r="6">
@@ -839,7 +839,7 @@
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>enterpriseCode</v>
+        <v>corporateCustomerId</v>
       </c>
       <c r="B9" t="str">
         <v/>
@@ -847,7 +847,7 @@
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>supplierId</v>
+        <v>partnerId</v>
       </c>
       <c r="B10" t="str">
         <v>NCC-001</v>
@@ -855,7 +855,7 @@
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>supplierName</v>
+        <v>partnerName</v>
       </c>
       <c r="B11" t="str">
         <v>NCC mẫu</v>

</xml_diff>